<commit_message>
feat(organization): 직원목록 엑셀다운로드 구현(RC_006)
- ws/organization/employee/download/list 신설(customerCard 엑셀다운로드와 동일 패턴)
- employeeList.js #saveExcelcs 클릭 핸들러 연결
- RC_006.xlsx 템플릿에 직원목록 컬럼 placeholder 채움(제목만 있던 상태)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/localcsms/web/admin-web/src/main/resources/RC_006.xlsx
+++ b/localcsms/web/admin-web/src/main/resources/RC_006.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>No.</t>
     <phoneticPr fontId="0" type="noConversion"/>
@@ -64,6 +64,30 @@
   <si>
     <t>마지막로그인일</t>
     <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>${excelData.emplName}</t>
+  </si>
+  <si>
+    <t>${excelData.companyName}</t>
+  </si>
+  <si>
+    <t>${excelData.loginId}</t>
+  </si>
+  <si>
+    <t>${excelData.mblPhoneNo}</t>
+  </si>
+  <si>
+    <t>${excelData.roleType}</t>
+  </si>
+  <si>
+    <t>${excelData.emplStatus}</t>
+  </si>
+  <si>
+    <t>${excelData.regDate}</t>
+  </si>
+  <si>
+    <t>${excelData.lastLoginDate}</t>
   </si>
 </sst>
 </file>
@@ -579,14 +603,30 @@
       <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
+      <c r="C5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>18</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>